<commit_message>
new labs added and changes made
</commit_message>
<xml_diff>
--- a/lab_07_2nd_part.xlsx
+++ b/lab_07_2nd_part.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Shreena\OneDrive\Desktop\office automation tools\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ce99177b26c586f9/Desktop/office automation tools/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4C22DBA-82DF-49F9-9211-D02834A74A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{C4C22DBA-82DF-49F9-9211-D02834A74A68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3DAAAA1-DBB7-461A-8E7E-EAFD8F5191E0}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{F7B7771D-CFAB-42C5-8108-B5833BE3195B}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{F7B7771D-CFAB-42C5-8108-B5833BE3195B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -719,13 +718,4 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D43505AF-B83E-4385-B1EE-86D96B5824F6}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <sheetData/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>